<commit_message>
fixed double barrel questions
</commit_message>
<xml_diff>
--- a/BINA NUSA Index Questions.xlsx
+++ b/BINA NUSA Index Questions.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Brilly Work\Downloads\Paper DT December 2025\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\github_repo\dti-deck\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7DC0EAFF-BAB9-4B21-AD0A-FF24D0FAD0B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{471AF214-D28D-4B19-8E99-17E29DD2E12C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BINA" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2083" uniqueCount="1206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2083" uniqueCount="1207">
   <si>
     <t>Index</t>
   </si>
@@ -3691,6 +3691,9 @@
     <t>1) Manajemen berniat memperluas skala inisiatif digital dalam beberapa tahun ke depan.
 2) Transformasi digital sering dibahas sebagai prioritas masa depan organisasi.
 3) Ada komitmen untuk menjadikan digital sebagai salah satu pilar utama strategi bisnis.</t>
+  </si>
+  <si>
+    <t>I3</t>
   </si>
 </sst>
 </file>
@@ -4508,7 +4511,7 @@
         <v>55</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>70</v>
+        <v>1206</v>
       </c>
       <c r="E18" s="5" t="s">
         <v>71</v>
@@ -4537,7 +4540,7 @@
         <v>55</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>70</v>
+        <v>1206</v>
       </c>
       <c r="E19" s="5" t="s">
         <v>71</v>
@@ -4566,7 +4569,7 @@
         <v>55</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="E20" s="5" t="s">
         <v>78</v>
@@ -4595,7 +4598,7 @@
         <v>55</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="E21" s="5" t="s">
         <v>78</v>
@@ -4624,7 +4627,7 @@
         <v>55</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="E22" s="5" t="s">
         <v>85</v>
@@ -4653,7 +4656,7 @@
         <v>55</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="E23" s="5" t="s">
         <v>85</v>

</xml_diff>